<commit_message>
update prep runway dashboards
</commit_message>
<xml_diff>
--- a/frontend/public/prep-runway/prep-runway-google-sheets-2026-05-22.xlsx
+++ b/frontend/public/prep-runway/prep-runway-google-sheets-2026-05-22.xlsx
@@ -19,12 +19,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Daily Ledger'!$A$1:$U$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Meal Timing'!$A$1:$J$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Training'!$A$1:$O$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sleep Recovery'!$A$1:$O$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Meal Timing'!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Training'!$A$1:$O$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sleep Recovery'!$A$1:$O$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Feedback Loop'!$A$1:$J$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Runway Narrative'!$A$1:$M$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Food Log Raw'!$A$1:$N$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Food Log Raw'!$A$1:$N$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'MacroFactor Daily'!$A$1:$Q$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -205,8 +205,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MealTiming" displayName="MealTiming" ref="A1:J22" headerRowCount="1">
-  <autoFilter ref="A1:J22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MealTiming" displayName="MealTiming" ref="A1:J23" headerRowCount="1">
+  <autoFilter ref="A1:J23"/>
   <tableColumns count="10">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="day"/>
@@ -224,8 +224,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Training" displayName="Training" ref="A1:O19" headerRowCount="1">
-  <autoFilter ref="A1:O19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Training" displayName="Training" ref="A1:O23" headerRowCount="1">
+  <autoFilter ref="A1:O23"/>
   <tableColumns count="15">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="session_order"/>
@@ -248,8 +248,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SleepRecovery" displayName="SleepRecovery" ref="A1:O6" headerRowCount="1">
-  <autoFilter ref="A1:O6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SleepRecovery" displayName="SleepRecovery" ref="A1:O7" headerRowCount="1">
+  <autoFilter ref="A1:O7"/>
   <tableColumns count="15">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="day"/>
@@ -313,8 +313,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FoodLogRaw" displayName="FoodLogRaw" ref="A1:N29" headerRowCount="1">
-  <autoFilter ref="A1:N29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="FoodLogRaw" displayName="FoodLogRaw" ref="A1:N35" headerRowCount="1">
+  <autoFilter ref="A1:N35"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Time"/>
@@ -673,7 +673,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22 11:01 AM</t>
+          <t>2026-05-22 09:18 PM</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>963 cal / 174P / 11.8F / 35.5C</t>
+          <t>917 cal / 162P / 12.7F / 34.9C</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Current check-in</t>
+          <t>Aggressive/Recoverable D2</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
@@ -1342,28 +1342,66 @@
       <c r="E7" s="5" t="n">
         <v>-0.3</v>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr"/>
-      <c r="O7" s="5" t="inlineStr"/>
-      <c r="P7" s="5" t="inlineStr"/>
-      <c r="Q7" s="5" t="inlineStr"/>
-      <c r="R7" s="5" t="inlineStr"/>
-      <c r="S7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>7h25m</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>7h25m</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>688</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Stair 50:37 + Stair 50:00</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Pull 108:07</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>11987</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>1901</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>1650</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="S7" s="5" t="n">
+        <v>116.6</v>
+      </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>flat-ish but still down 10.6 lb from 5/17 — Use marker-led cardio and GI-friendly protein.</t>
+          <t>Workout/day totals locked; macros still partial at 688 cal / 101P. PM Stair added and day became high-output.</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>cleanup-feedback-loop-may17-jun1-2026.csv; user-reported 158.4 lb</t>
+          <t>MacroFactor export 2026-05-22 17:42 + Claude full-session Apple Health pull pasted in Codex chat 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2342,31 +2380,83 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>11:33a</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>No food logged in export yet</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr"/>
+          <t>Chicken + egg whites + avocado + turkey bacon</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>451</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Use feedback loop today.</t>
+          <t>Whole-food base; better GI structure than all-powder days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>3:17p</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Banana + chocolate nutrition shake</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>237</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Pre-lift fuel; controlled carb bump before pull day.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J22"/>
+  <autoFilter ref="A1:J23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2380,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2395,7 +2485,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
     <col width="48" customWidth="1" min="14" max="14"/>
     <col width="48" customWidth="1" min="15" max="15"/>
   </cols>
@@ -3605,8 +3695,258 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>7:03 AM</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>7:54 AM</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>StairMaster</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>50:37</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>518</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>518</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>144</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Z3 moderate</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>AM stair was controlled lower-HR output than Wed/Thu; useful anchor without spiking too hard.</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Claude Apple Health pull pasted in Codex chat 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>3:43 PM</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>3:44 PM</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Warmup</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>1:16</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>97</v>
+      </c>
+      <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Z1/Z2</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Raw context only; excluded from readable ledger per user preference.</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Claude Apple Health pull pasted in Codex chat 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>3:45 PM</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>5:33 PM</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Pull day</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>108:07</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>606</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>510</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>111</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>146</v>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Z2/Z3</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Long pull day; lower HR than Thu but user felt deficit around minute 60, so do not interpret the lower burn as room to add punishment volume.</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>MacroFactor workout log + Claude full-session Apple Health pull pasted in Codex chat 2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>5:35 PM</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>6:25 PM</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>StairMaster</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>50:00</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>528</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>528</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>132</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Z3 moderate with spike</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>PM StairMaster matched AM average effort but peaked at 175 after the long pull day; useful output, but this is a hard post-lift spike and should count as high stress.</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>Claude full-session Apple Health pull pasted in Codex chat 2026-05-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O19"/>
+  <autoFilter ref="A1:O23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3620,7 +3960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4074,8 +4414,81 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>11:58p Thu</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>7:29a</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>7h25m</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>4h38m</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>2h10m</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>35m</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>116.6</v>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Good recovery marker day before another high-output training day.</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>Claude full-session Apple Health pull pasted in Codex chat 2026-05-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O6"/>
+  <autoFilter ref="A1:O7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4096,7 +4509,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
@@ -4417,32 +4830,32 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>GI check pending</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>stool check pending</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>deficit felt during lift after ~60m</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>needs check-in</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>needs check-in</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>needs check-in</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>needs check-in</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>needs check-in</t>
-        </is>
-      </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>needs check-in</t>
+          <t>pull day plus two StairMasters; PM stair peaked 175</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -4452,7 +4865,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Use marker-led cardio and GI-friendly protein.</t>
+          <t>Do not add more training today. Finish final macros and use Sat AM weight/RHR/HRV/sleep to decide whether to keep aggressive or pull back.</t>
         </is>
       </c>
     </row>
@@ -4856,7 +5269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6375,8 +6788,308 @@
       </c>
       <c r="N29" s="5" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>11:33 AM</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Chicken Breasts</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>oz</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>28.35</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>146</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="M30" s="5" t="n">
+        <v>473.2</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>11:33 AM</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Egg Whites</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="n">
+        <v>375</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>375</v>
+      </c>
+      <c r="N31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>11:33 AM</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Organic Avocado Mash</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>container</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>220</v>
+      </c>
+      <c r="M32" s="5" t="n">
+        <v>270.2</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>11:33 AM</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Uncured Turkey Bacon Turkey Thighs Chopped and Formed</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>serving</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="5" t="inlineStr"/>
+      <c r="L33" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>03:17 PM</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Banana, Fresh</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L34" s="5" t="inlineStr"/>
+      <c r="M34" s="5" t="n">
+        <v>322.7</v>
+      </c>
+      <c r="N34" s="5" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>03:17 PM</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Chocolate Nutrition Shake</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="M35" s="5" t="n">
+        <v>460</v>
+      </c>
+      <c r="N35" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N29"/>
+  <autoFilter ref="A1:N35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6806,21 +7519,45 @@
         <v>151.42</v>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="n">
+        <v>688</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>150</v>
+      </c>
       <c r="M8" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="N8" s="5" t="inlineStr"/>
-      <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
-      <c r="Q8" s="5" t="inlineStr"/>
+        <v>8032</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>1256.3</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>2061.1</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>42.2</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q8"/>

</xml_diff>